<commit_message>
El problema es que mai acabo i faig, comit sino que sempre començo coses noves
</commit_message>
<xml_diff>
--- a/data/punts/punts-mesura-ste.xlsx
+++ b/data/punts/punts-mesura-ste.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ArnauCoronado\Documents_local\vapor\data\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ArnauCoronado\Documents_local\euromed\sxs\data\punts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6C46708-9BF6-427A-9957-65B8C2222745}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BCA5F11-EA93-464B-9CDC-1D250A485231}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{4CA701B3-5EB8-45D8-B6BB-1F057196BE44}"/>
   </bookViews>
@@ -666,10 +666,10 @@
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
-        <v>1514</v>
+        <v>1458</v>
       </c>
       <c r="B2" s="1">
-        <v>854</v>
+        <v>879</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>38</v>
@@ -724,10 +724,10 @@
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
-        <v>1104</v>
+        <v>1088</v>
       </c>
       <c r="B3" s="1">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>39</v>
@@ -782,10 +782,10 @@
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
-        <v>1154</v>
+        <v>1141</v>
       </c>
       <c r="B4" s="1">
-        <v>514</v>
+        <v>544.5</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>40</v>
@@ -840,10 +840,10 @@
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
-        <v>1143</v>
+        <v>1099.5</v>
       </c>
       <c r="B5" s="1">
-        <v>323</v>
+        <v>282</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>41</v>
@@ -895,10 +895,10 @@
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
-        <v>843</v>
+        <v>952.5</v>
       </c>
       <c r="B6" s="1">
-        <v>908</v>
+        <v>920</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>42</v>
@@ -953,10 +953,10 @@
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
-        <v>903</v>
+        <v>966.5</v>
       </c>
       <c r="B7" s="1">
-        <v>908</v>
+        <v>920</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>43</v>
@@ -1011,10 +1011,10 @@
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
-        <v>940</v>
+        <v>938</v>
       </c>
       <c r="B8" s="1">
-        <v>908</v>
+        <v>986.5</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>44</v>
@@ -1069,10 +1069,10 @@
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="B9" s="1">
-        <v>509</v>
+        <v>553</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>45</v>
@@ -1127,10 +1127,10 @@
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
-        <v>745</v>
+        <v>647</v>
       </c>
       <c r="B10" s="1">
-        <v>514</v>
+        <v>580</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>46</v>
@@ -1182,10 +1182,10 @@
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
-        <v>352</v>
+        <v>432.5</v>
       </c>
       <c r="B11" s="1">
-        <v>749</v>
+        <v>689</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>47</v>
@@ -1240,10 +1240,10 @@
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
-        <v>265</v>
+        <v>395.5</v>
       </c>
       <c r="B12" s="1">
-        <v>1333</v>
+        <v>1312</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>48</v>

</xml_diff>

<commit_message>
gui actualitzada amb mapa en html
</commit_message>
<xml_diff>
--- a/data/punts/punts-mesura-ste.xlsx
+++ b/data/punts/punts-mesura-ste.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ArnauCoronado\Documents_local\euromed\sxs\data\punts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E26F2EA-8922-460B-A2C3-B1662544D9BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{680C8061-D588-46BC-AFDA-775E98120C72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{4CA701B3-5EB8-45D8-B6BB-1F057196BE44}"/>
   </bookViews>
@@ -639,7 +639,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P29"/>
+  <dimension ref="A1:P28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="8.88671875" style="1"/>
@@ -742,7 +742,7 @@
         <v>46</v>
       </c>
       <c r="L2" s="3">
-        <f>PI()*(((I2-2*J2)*10^-3)^2)/4</f>
+        <f t="shared" ref="L2:L12" si="0">PI()*(((I2-2*J2)*10^-3)^2)/4</f>
         <v>5.319729526158304E-3</v>
       </c>
       <c r="M2" s="4">
@@ -796,22 +796,22 @@
         <v>46</v>
       </c>
       <c r="L3" s="3">
-        <f>PI()*(((I3-2*J3)*10^-3)^2)/4</f>
+        <f t="shared" si="0"/>
         <v>5.319729526158304E-3</v>
       </c>
       <c r="M3" s="4">
         <v>7.5</v>
       </c>
       <c r="N3" s="3">
-        <f t="shared" ref="N3:N12" si="0">M3*L3</f>
+        <f t="shared" ref="N3:N12" si="1">M3*L3</f>
         <v>3.9897971446187279E-2</v>
       </c>
       <c r="O3" s="3">
-        <f t="shared" ref="O3:O12" si="1">N3*3600</f>
+        <f t="shared" ref="O3:O12" si="2">N3*3600</f>
         <v>143.6326972062742</v>
       </c>
       <c r="P3" s="3">
-        <f t="shared" ref="P3:P12" si="2">O3*4.3</f>
+        <f t="shared" ref="P3:P12" si="3">O3*4.3</f>
         <v>617.62059798697908</v>
       </c>
     </row>
@@ -850,22 +850,22 @@
         <v>46</v>
       </c>
       <c r="L4" s="3">
-        <f>PI()*(((I4-2*J4)*10^-3)^2)/4</f>
+        <f t="shared" si="0"/>
         <v>1.4186929768786934E-2</v>
       </c>
       <c r="M4" s="4">
         <v>2.2999999999999998</v>
       </c>
       <c r="N4" s="3">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>3.2629938468209947E-2</v>
       </c>
       <c r="O4" s="3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>117.46777848555581</v>
       </c>
       <c r="P4" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>505.11144748788996</v>
       </c>
     </row>
@@ -904,7 +904,7 @@
         <v>46</v>
       </c>
       <c r="L5" s="3">
-        <f>PI()*(((I5-2*J5)*10^-3)^2)/4</f>
+        <f t="shared" si="0"/>
         <v>4.5364597917836608E-3</v>
       </c>
       <c r="M5" s="4" t="s">
@@ -955,22 +955,22 @@
         <v>46</v>
       </c>
       <c r="L6" s="3">
-        <f>PI()*(((I6-2*J6)*10^-3)^2)/4</f>
+        <f t="shared" si="0"/>
         <v>2.8557784079478277E-3</v>
       </c>
       <c r="M6" s="4">
         <v>13.54</v>
       </c>
       <c r="N6" s="3">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>3.8667239643613585E-2</v>
       </c>
       <c r="O6" s="3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>139.20206271700891</v>
       </c>
       <c r="P6" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>598.56886968313836</v>
       </c>
     </row>
@@ -1009,22 +1009,22 @@
         <v>46</v>
       </c>
       <c r="L7" s="3">
-        <f>PI()*(((I7-2*J7)*10^-3)^2)/4</f>
+        <f t="shared" si="0"/>
         <v>1.3074051987179279E-3</v>
       </c>
       <c r="M7" s="4">
         <v>0.2</v>
       </c>
       <c r="N7" s="3">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2.6148103974358558E-4</v>
       </c>
       <c r="O7" s="3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.94133174307690803</v>
       </c>
       <c r="P7" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>4.0477264952307044</v>
       </c>
     </row>
@@ -1063,22 +1063,22 @@
         <v>46</v>
       </c>
       <c r="L8" s="3">
-        <f>PI()*(((I8-2*J8)*10^-3)^2)/4</f>
+        <f t="shared" si="0"/>
         <v>1.0207034531513238E-2</v>
       </c>
       <c r="M8" s="4">
         <v>7.5</v>
       </c>
       <c r="N8" s="3">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>7.6552758986349292E-2</v>
       </c>
       <c r="O8" s="3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>275.58993235085745</v>
       </c>
       <c r="P8" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1185.0367091086871</v>
       </c>
     </row>
@@ -1117,22 +1117,22 @@
         <v>46</v>
       </c>
       <c r="L9" s="3">
-        <f>PI()*(((I9-2*J9)*10^-3)^2)/4</f>
+        <f t="shared" si="0"/>
         <v>2.3671979184615426E-3</v>
       </c>
       <c r="M9" s="4">
         <v>2</v>
       </c>
       <c r="N9" s="3">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>4.7343958369230853E-3</v>
       </c>
       <c r="O9" s="3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>17.043825012923108</v>
       </c>
       <c r="P9" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>73.288447555569363</v>
       </c>
     </row>
@@ -1171,7 +1171,7 @@
         <v>46</v>
       </c>
       <c r="L10" s="3">
-        <f>PI()*(((I10-2*J10)*10^-3)^2)/4</f>
+        <f t="shared" si="0"/>
         <v>1.4725351625722418E-3</v>
       </c>
       <c r="M10" s="4" t="s">
@@ -1222,22 +1222,22 @@
         <v>46</v>
       </c>
       <c r="L11" s="3">
-        <f>PI()*(((I11-2*J11)*10^-3)^2)/4</f>
+        <f t="shared" si="0"/>
         <v>3.5890811111671224E-3</v>
       </c>
       <c r="M11" s="4">
         <v>0.1</v>
       </c>
       <c r="N11" s="3">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>3.5890811111671225E-4</v>
       </c>
       <c r="O11" s="3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1.2920692000201641</v>
       </c>
       <c r="P11" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>5.5558975600867058</v>
       </c>
     </row>
@@ -1276,22 +1276,22 @@
         <v>46</v>
       </c>
       <c r="L12" s="3">
-        <f>PI()*(((I12-2*J12)*10^-3)^2)/4</f>
+        <f t="shared" si="0"/>
         <v>3.8704735651491607E-3</v>
       </c>
       <c r="M12" s="4">
         <v>1.6</v>
       </c>
       <c r="N12" s="3">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6.1927577042386571E-3</v>
       </c>
       <c r="O12" s="3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>22.293927735259164</v>
       </c>
       <c r="P12" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>95.863889261614403</v>
       </c>
     </row>
@@ -1407,15 +1407,7 @@
       <c r="J28" s="5"/>
       <c r="M28" s="5"/>
     </row>
-    <row r="29" spans="6:13" x14ac:dyDescent="0.3">
-      <c r="F29" s="5"/>
-      <c r="G29" s="5"/>
-      <c r="I29" s="5"/>
-      <c r="J29" s="5"/>
-      <c r="M29" s="5"/>
-    </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="i82pyk6g/nclq841DWlAoSd0VpLuJ09FkNrJENEDkV8KiHmrVm2pbdnxOvLz4OciGGLKfaGIWnBbdyPjV5W8bA==" saltValue="9Jhl/0bmR6iS7aXe+HwzQg==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <autoFilter ref="A1:N1" xr:uid="{80D9219E-119C-467C-9531-507D24E0A5C1}"/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>